<commit_message>
Update DCA tracker and backtest outputs
</commit_message>
<xml_diff>
--- a/strategies/constant_value/定投追踪记录.xlsx
+++ b/strategies/constant_value/定投追踪记录.xlsx
@@ -1151,8 +1151,14 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="n"/>
-      <c r="B7" s="33" t="n"/>
+      <c r="A7" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
       <c r="C7" s="7">
         <f>IFERROR(SUMIF(沪深300!$B$5:$B$1000,A7,沪深300!$L$5:$L$1000),"")</f>
         <v/>
@@ -1173,7 +1179,9 @@
         <f>IFERROR(IF(M7="增量阶段",H7,SUMPRODUCT(MAX(C7,0),1)+SUMPRODUCT(MAX(D7,0),1)+SUMPRODUCT(MAX(E7,0),1)+SUMPRODUCT(MAX(F7,0),1)),"")</f>
         <v/>
       </c>
-      <c r="H7" s="17" t="n"/>
+      <c r="H7" s="17" t="n">
+        <v>0</v>
+      </c>
       <c r="I7" s="7">
         <f>IFERROR(MAX(-C7,0)+MAX(-D7,0)+MAX(-E7,0)+MAX(-F7,0),"")</f>
         <v/>
@@ -6137,19 +6145,31 @@
       <c r="Q6" s="32" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="33" t="n"/>
-      <c r="B7" s="15" t="n"/>
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>3</v>
+      </c>
       <c r="C7" s="7">
         <f>IFERROR(参数配置!$C$5*(B7-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D7" s="27" t="n"/>
-      <c r="E7" s="27" t="n"/>
+      <c r="D7" s="27" t="n">
+        <v>4.828</v>
+      </c>
+      <c r="E7" s="27" t="n">
+        <v>4.4239</v>
+      </c>
       <c r="F7" s="28">
         <f>IFERROR((D7-E7)/E7,"")</f>
         <v/>
       </c>
-      <c r="G7" s="27" t="n"/>
+      <c r="G7" s="27" t="n">
+        <v>600</v>
+      </c>
       <c r="H7" s="7">
         <f>IFERROR(G7*D7,"")</f>
         <v/>
@@ -6166,8 +6186,12 @@
         <f>IFERROR(I7,"")</f>
         <v/>
       </c>
-      <c r="L7" s="17" t="n"/>
-      <c r="M7" s="27" t="n"/>
+      <c r="L7" s="17" t="n">
+        <v>1448.4</v>
+      </c>
+      <c r="M7" s="27" t="n">
+        <v>300</v>
+      </c>
       <c r="N7" s="31">
         <f>IFERROR(G7+M7,"")</f>
         <v/>
@@ -10946,19 +10970,31 @@
       <c r="Q6" s="32" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="33" t="n"/>
-      <c r="B7" s="15" t="n"/>
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>3</v>
+      </c>
       <c r="C7" s="7">
         <f>IFERROR(参数配置!$C$6*(B7-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D7" s="27" t="n"/>
-      <c r="E7" s="27" t="n"/>
+      <c r="D7" s="27" t="n">
+        <v>8.576000000000001</v>
+      </c>
+      <c r="E7" s="27" t="n">
+        <v>7.2287</v>
+      </c>
       <c r="F7" s="28">
         <f>IFERROR((D7-E7)/E7,"")</f>
         <v/>
       </c>
-      <c r="G7" s="27" t="n"/>
+      <c r="G7" s="27" t="n">
+        <v>300</v>
+      </c>
       <c r="H7" s="7">
         <f>IFERROR(G7*D7,"")</f>
         <v/>
@@ -10975,8 +11011,12 @@
         <f>IFERROR(I7,"")</f>
         <v/>
       </c>
-      <c r="L7" s="17" t="n"/>
-      <c r="M7" s="27" t="n"/>
+      <c r="L7" s="17" t="n">
+        <v>1715.2</v>
+      </c>
+      <c r="M7" s="27" t="n">
+        <v>200</v>
+      </c>
       <c r="N7" s="31">
         <f>IFERROR(G7+M7,"")</f>
         <v/>
@@ -15755,19 +15795,31 @@
       <c r="Q6" s="32" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="33" t="n"/>
-      <c r="B7" s="15" t="n"/>
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>3</v>
+      </c>
       <c r="C7" s="7">
         <f>IFERROR(参数配置!$C$7*(B7-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D7" s="27" t="n"/>
-      <c r="E7" s="27" t="n"/>
+      <c r="D7" s="27" t="n">
+        <v>1.504</v>
+      </c>
+      <c r="E7" s="27" t="n">
+        <v>1.5507</v>
+      </c>
       <c r="F7" s="28">
         <f>IFERROR((D7-E7)/E7,"")</f>
         <v/>
       </c>
-      <c r="G7" s="27" t="n"/>
+      <c r="G7" s="27" t="n">
+        <v>700</v>
+      </c>
       <c r="H7" s="7">
         <f>IFERROR(G7*D7,"")</f>
         <v/>
@@ -15784,8 +15836,12 @@
         <f>IFERROR(I7,"")</f>
         <v/>
       </c>
-      <c r="L7" s="17" t="n"/>
-      <c r="M7" s="27" t="n"/>
+      <c r="L7" s="17" t="n">
+        <v>752</v>
+      </c>
+      <c r="M7" s="27" t="n">
+        <v>500</v>
+      </c>
       <c r="N7" s="31">
         <f>IFERROR(G7+M7,"")</f>
         <v/>
@@ -20564,19 +20620,31 @@
       <c r="Q6" s="32" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="33" t="n"/>
-      <c r="B7" s="15" t="n"/>
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>3</v>
+      </c>
       <c r="C7" s="7">
         <f>IFERROR(参数配置!$C$8*(B7-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D7" s="27" t="n"/>
-      <c r="E7" s="27" t="n"/>
+      <c r="D7" s="27" t="n">
+        <v>2.124</v>
+      </c>
+      <c r="E7" s="27" t="n">
+        <v>1.7868</v>
+      </c>
       <c r="F7" s="28">
         <f>IFERROR((D7-E7)/E7,"")</f>
         <v/>
       </c>
-      <c r="G7" s="27" t="n"/>
+      <c r="G7" s="27" t="n">
+        <v>2300</v>
+      </c>
       <c r="H7" s="7">
         <f>IFERROR(G7*D7,"")</f>
         <v/>
@@ -20593,8 +20661,12 @@
         <f>IFERROR(I7,"")</f>
         <v/>
       </c>
-      <c r="L7" s="17" t="n"/>
-      <c r="M7" s="27" t="n"/>
+      <c r="L7" s="17" t="n">
+        <v>2336.4</v>
+      </c>
+      <c r="M7" s="27" t="n">
+        <v>1100</v>
+      </c>
       <c r="N7" s="31">
         <f>IFERROR(G7+M7,"")</f>
         <v/>

</xml_diff>

<commit_message>
Record DCA period 4
</commit_message>
<xml_diff>
--- a/strategies/constant_value/定投追踪记录.xlsx
+++ b/strategies/constant_value/定投追踪记录.xlsx
@@ -1204,8 +1204,14 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="n"/>
-      <c r="B8" s="33" t="n"/>
+      <c r="A8" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
       <c r="C8" s="7">
         <f>IFERROR(SUMIF(沪深300!$B$5:$B$1000,A8,沪深300!$L$5:$L$1000),"")</f>
         <v/>
@@ -1226,7 +1232,9 @@
         <f>IFERROR(IF(M8="增量阶段",H8,SUMPRODUCT(MAX(C8,0),1)+SUMPRODUCT(MAX(D8,0),1)+SUMPRODUCT(MAX(E8,0),1)+SUMPRODUCT(MAX(F8,0),1)),"")</f>
         <v/>
       </c>
-      <c r="H8" s="17" t="n"/>
+      <c r="H8" s="17" t="n">
+        <v>0</v>
+      </c>
       <c r="I8" s="7">
         <f>IFERROR(MAX(-C8,0)+MAX(-D8,0)+MAX(-E8,0)+MAX(-F8,0),"")</f>
         <v/>
@@ -6207,19 +6215,31 @@
       <c r="Q7" s="32" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="33" t="n"/>
-      <c r="B8" s="15" t="n"/>
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="n">
+        <v>4</v>
+      </c>
       <c r="C8" s="7">
         <f>IFERROR(参数配置!$C$5*(B8-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D8" s="27" t="n"/>
-      <c r="E8" s="27" t="n"/>
+      <c r="D8" s="27" t="n">
+        <v>4.91</v>
+      </c>
+      <c r="E8" s="27" t="n">
+        <v>4.46819947052002</v>
+      </c>
       <c r="F8" s="28">
         <f>IFERROR((D8-E8)/E8,"")</f>
         <v/>
       </c>
-      <c r="G8" s="27" t="n"/>
+      <c r="G8" s="27" t="n">
+        <v>900</v>
+      </c>
       <c r="H8" s="7">
         <f>IFERROR(G8*D8,"")</f>
         <v/>
@@ -6236,8 +6256,12 @@
         <f>IFERROR(I8,"")</f>
         <v/>
       </c>
-      <c r="L8" s="17" t="n"/>
-      <c r="M8" s="27" t="n"/>
+      <c r="L8" s="17" t="n">
+        <v>1473</v>
+      </c>
+      <c r="M8" s="27" t="n">
+        <v>300</v>
+      </c>
       <c r="N8" s="31">
         <f>IFERROR(G8+M8,"")</f>
         <v/>
@@ -11032,19 +11056,31 @@
       <c r="Q7" s="32" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="33" t="n"/>
-      <c r="B8" s="15" t="n"/>
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="n">
+        <v>4</v>
+      </c>
       <c r="C8" s="7">
         <f>IFERROR(参数配置!$C$6*(B8-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D8" s="27" t="n"/>
-      <c r="E8" s="27" t="n"/>
+      <c r="D8" s="27" t="n">
+        <v>8.333</v>
+      </c>
+      <c r="E8" s="27" t="n">
+        <v>7.342891065597534</v>
+      </c>
       <c r="F8" s="28">
         <f>IFERROR((D8-E8)/E8,"")</f>
         <v/>
       </c>
-      <c r="G8" s="27" t="n"/>
+      <c r="G8" s="27" t="n">
+        <v>500</v>
+      </c>
       <c r="H8" s="7">
         <f>IFERROR(G8*D8,"")</f>
         <v/>
@@ -11061,8 +11097,12 @@
         <f>IFERROR(I8,"")</f>
         <v/>
       </c>
-      <c r="L8" s="17" t="n"/>
-      <c r="M8" s="27" t="n"/>
+      <c r="L8" s="17" t="n">
+        <v>2499.9</v>
+      </c>
+      <c r="M8" s="27" t="n">
+        <v>300</v>
+      </c>
       <c r="N8" s="31">
         <f>IFERROR(G8+M8,"")</f>
         <v/>
@@ -15857,19 +15897,31 @@
       <c r="Q7" s="32" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="33" t="n"/>
-      <c r="B8" s="15" t="n"/>
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="n">
+        <v>4</v>
+      </c>
       <c r="C8" s="7">
         <f>IFERROR(参数配置!$C$7*(B8-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D8" s="27" t="n"/>
-      <c r="E8" s="27" t="n"/>
+      <c r="D8" s="27" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="E8" s="27" t="n">
+        <v>1.553168001651764</v>
+      </c>
       <c r="F8" s="28">
         <f>IFERROR((D8-E8)/E8,"")</f>
         <v/>
       </c>
-      <c r="G8" s="27" t="n"/>
+      <c r="G8" s="27" t="n">
+        <v>1200</v>
+      </c>
       <c r="H8" s="7">
         <f>IFERROR(G8*D8,"")</f>
         <v/>
@@ -15886,8 +15938,12 @@
         <f>IFERROR(I8,"")</f>
         <v/>
       </c>
-      <c r="L8" s="17" t="n"/>
-      <c r="M8" s="27" t="n"/>
+      <c r="L8" s="17" t="n">
+        <v>740</v>
+      </c>
+      <c r="M8" s="27" t="n">
+        <v>500</v>
+      </c>
       <c r="N8" s="31">
         <f>IFERROR(G8+M8,"")</f>
         <v/>
@@ -20682,19 +20738,31 @@
       <c r="Q7" s="32" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="33" t="n"/>
-      <c r="B8" s="15" t="n"/>
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="n">
+        <v>4</v>
+      </c>
       <c r="C8" s="7">
         <f>IFERROR(参数配置!$C$8*(B8-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D8" s="27" t="n"/>
-      <c r="E8" s="27" t="n"/>
+      <c r="D8" s="27" t="n">
+        <v>2.214</v>
+      </c>
+      <c r="E8" s="27" t="n">
+        <v>1.814727995872498</v>
+      </c>
       <c r="F8" s="28">
         <f>IFERROR((D8-E8)/E8,"")</f>
         <v/>
       </c>
-      <c r="G8" s="27" t="n"/>
+      <c r="G8" s="27" t="n">
+        <v>3400</v>
+      </c>
       <c r="H8" s="7">
         <f>IFERROR(G8*D8,"")</f>
         <v/>
@@ -20711,8 +20779,12 @@
         <f>IFERROR(I8,"")</f>
         <v/>
       </c>
-      <c r="L8" s="17" t="n"/>
-      <c r="M8" s="27" t="n"/>
+      <c r="L8" s="17" t="n">
+        <v>2214</v>
+      </c>
+      <c r="M8" s="27" t="n">
+        <v>1000</v>
+      </c>
       <c r="N8" s="31">
         <f>IFERROR(G8+M8,"")</f>
         <v/>

</xml_diff>

<commit_message>
Record DCA period 5 and harden dca-update skill.
Capture holiday-period trades including Nasdaq halt, and fix skill scripts so G column correctly chains from prior N shares.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/strategies/constant_value/定投追踪记录.xlsx
+++ b/strategies/constant_value/定投追踪记录.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总看板" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每期汇总" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数配置" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="沪深300" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="恒生指数" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="纳指100" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="汇总看板" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="每期汇总" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="参数配置" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="沪深300" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="中证500" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="恒生指数" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="纳指100" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1257,8 +1257,14 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="n"/>
-      <c r="B9" s="33" t="n"/>
+      <c r="A9" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
       <c r="C9" s="7">
         <f>IFERROR(SUMIF(沪深300!$B$5:$B$1000,A9,沪深300!$L$5:$L$1000),"")</f>
         <v/>
@@ -1279,7 +1285,9 @@
         <f>IFERROR(IF(M9="增量阶段",H9,SUMPRODUCT(MAX(C9,0),1)+SUMPRODUCT(MAX(D9,0),1)+SUMPRODUCT(MAX(E9,0),1)+SUMPRODUCT(MAX(F9,0),1)),"")</f>
         <v/>
       </c>
-      <c r="H9" s="17" t="n"/>
+      <c r="H9" s="17" t="n">
+        <v>0</v>
+      </c>
       <c r="I9" s="7">
         <f>IFERROR(MAX(-C9,0)+MAX(-D9,0)+MAX(-E9,0)+MAX(-F9,0),"")</f>
         <v/>
@@ -6277,19 +6285,31 @@
       <c r="Q8" s="32" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="33" t="n"/>
-      <c r="B9" s="15" t="n"/>
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>5</v>
+      </c>
       <c r="C9" s="7">
         <f>IFERROR(参数配置!$C$5*(B9-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D9" s="27" t="n"/>
-      <c r="E9" s="27" t="n"/>
+      <c r="D9" s="27" t="n">
+        <v>4.975</v>
+      </c>
+      <c r="E9" s="27" t="n">
+        <v>4.46819947052002</v>
+      </c>
       <c r="F9" s="28">
         <f>IFERROR((D9-E9)/E9,"")</f>
         <v/>
       </c>
-      <c r="G9" s="27" t="n"/>
+      <c r="G9" s="27" t="n">
+        <v>1200</v>
+      </c>
       <c r="H9" s="7">
         <f>IFERROR(G9*D9,"")</f>
         <v/>
@@ -6306,8 +6326,12 @@
         <f>IFERROR(I9,"")</f>
         <v/>
       </c>
-      <c r="L9" s="17" t="n"/>
-      <c r="M9" s="27" t="n"/>
+      <c r="L9" s="17" t="n">
+        <v>1492.5</v>
+      </c>
+      <c r="M9" s="27" t="n">
+        <v>300</v>
+      </c>
       <c r="N9" s="31">
         <f>IFERROR(G9+M9,"")</f>
         <v/>
@@ -11118,19 +11142,31 @@
       <c r="Q8" s="32" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="33" t="n"/>
-      <c r="B9" s="15" t="n"/>
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>5</v>
+      </c>
       <c r="C9" s="7">
         <f>IFERROR(参数配置!$C$6*(B9-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D9" s="27" t="n"/>
-      <c r="E9" s="27" t="n"/>
+      <c r="D9" s="27" t="n">
+        <v>8.797000000000001</v>
+      </c>
+      <c r="E9" s="27" t="n">
+        <v>7.342891065597534</v>
+      </c>
       <c r="F9" s="28">
         <f>IFERROR((D9-E9)/E9,"")</f>
         <v/>
       </c>
-      <c r="G9" s="27" t="n"/>
+      <c r="G9" s="27" t="n">
+        <v>800</v>
+      </c>
       <c r="H9" s="7">
         <f>IFERROR(G9*D9,"")</f>
         <v/>
@@ -11147,8 +11183,12 @@
         <f>IFERROR(I9,"")</f>
         <v/>
       </c>
-      <c r="L9" s="17" t="n"/>
-      <c r="M9" s="27" t="n"/>
+      <c r="L9" s="17" t="n">
+        <v>879.7</v>
+      </c>
+      <c r="M9" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="N9" s="31">
         <f>IFERROR(G9+M9,"")</f>
         <v/>
@@ -15959,19 +15999,31 @@
       <c r="Q8" s="32" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="33" t="n"/>
-      <c r="B9" s="15" t="n"/>
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>5</v>
+      </c>
       <c r="C9" s="7">
         <f>IFERROR(参数配置!$C$7*(B9-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D9" s="27" t="n"/>
-      <c r="E9" s="27" t="n"/>
+      <c r="D9" s="27" t="n">
+        <v>1.412</v>
+      </c>
+      <c r="E9" s="27" t="n">
+        <v>1.553168001651764</v>
+      </c>
       <c r="F9" s="28">
         <f>IFERROR((D9-E9)/E9,"")</f>
         <v/>
       </c>
-      <c r="G9" s="27" t="n"/>
+      <c r="G9" s="27" t="n">
+        <v>1700</v>
+      </c>
       <c r="H9" s="7">
         <f>IFERROR(G9*D9,"")</f>
         <v/>
@@ -15988,8 +16040,12 @@
         <f>IFERROR(I9,"")</f>
         <v/>
       </c>
-      <c r="L9" s="17" t="n"/>
-      <c r="M9" s="27" t="n"/>
+      <c r="L9" s="17" t="n">
+        <v>706</v>
+      </c>
+      <c r="M9" s="27" t="n">
+        <v>500</v>
+      </c>
       <c r="N9" s="31">
         <f>IFERROR(G9+M9,"")</f>
         <v/>
@@ -20800,19 +20856,31 @@
       <c r="Q8" s="32" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="33" t="n"/>
-      <c r="B9" s="15" t="n"/>
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>5</v>
+      </c>
       <c r="C9" s="7">
         <f>IFERROR(参数配置!$C$8*(B9-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D9" s="27" t="n"/>
-      <c r="E9" s="27" t="n"/>
+      <c r="D9" s="27" t="n">
+        <v>2.214</v>
+      </c>
+      <c r="E9" s="27" t="n">
+        <v>1.814727995872498</v>
+      </c>
       <c r="F9" s="28">
         <f>IFERROR((D9-E9)/E9,"")</f>
         <v/>
       </c>
-      <c r="G9" s="27" t="n"/>
+      <c r="G9" s="27" t="n">
+        <v>4400</v>
+      </c>
       <c r="H9" s="7">
         <f>IFERROR(G9*D9,"")</f>
         <v/>
@@ -20829,8 +20897,12 @@
         <f>IFERROR(I9,"")</f>
         <v/>
       </c>
-      <c r="L9" s="17" t="n"/>
-      <c r="M9" s="27" t="n"/>
+      <c r="L9" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="N9" s="31">
         <f>IFERROR(G9+M9,"")</f>
         <v/>
@@ -20843,7 +20915,11 @@
         <f>IFERROR(-L9,"")</f>
         <v/>
       </c>
-      <c r="Q9" s="32" t="n"/>
+      <c r="Q9" s="32" t="inlineStr">
+        <is>
+          <t>停牌，本期暂停操作，目标市值照常增长</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="33" t="n"/>

</xml_diff>

<commit_message>
Record DCA period 6.
</commit_message>
<xml_diff>
--- a/strategies/constant_value/定投追踪记录.xlsx
+++ b/strategies/constant_value/定投追踪记录.xlsx
@@ -1310,8 +1310,14 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="n"/>
-      <c r="B10" s="33" t="n"/>
+      <c r="A10" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="33" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
       <c r="C10" s="7">
         <f>IFERROR(SUMIF(沪深300!$B$5:$B$1000,A10,沪深300!$L$5:$L$1000),"")</f>
         <v/>
@@ -1332,7 +1338,9 @@
         <f>IFERROR(IF(M10="增量阶段",H10,SUMPRODUCT(MAX(C10,0),1)+SUMPRODUCT(MAX(D10,0),1)+SUMPRODUCT(MAX(E10,0),1)+SUMPRODUCT(MAX(F10,0),1)),"")</f>
         <v/>
       </c>
-      <c r="H10" s="17" t="n"/>
+      <c r="H10" s="17" t="n">
+        <v>0</v>
+      </c>
       <c r="I10" s="7">
         <f>IFERROR(MAX(-C10,0)+MAX(-D10,0)+MAX(-E10,0)+MAX(-F10,0),"")</f>
         <v/>
@@ -6347,19 +6355,31 @@
       <c r="Q9" s="32" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="33" t="n"/>
-      <c r="B10" s="15" t="n"/>
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="n">
+        <v>6</v>
+      </c>
       <c r="C10" s="7">
         <f>IFERROR(参数配置!$C$5*(B10-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D10" s="27" t="n"/>
-      <c r="E10" s="27" t="n"/>
+      <c r="D10" s="27" t="n">
+        <v>4.852</v>
+      </c>
+      <c r="E10" s="27" t="n">
+        <v>4.46819947052002</v>
+      </c>
       <c r="F10" s="28">
         <f>IFERROR((D10-E10)/E10,"")</f>
         <v/>
       </c>
-      <c r="G10" s="27" t="n"/>
+      <c r="G10" s="27" t="n">
+        <v>1500</v>
+      </c>
       <c r="H10" s="7">
         <f>IFERROR(G10*D10,"")</f>
         <v/>
@@ -6376,8 +6396,12 @@
         <f>IFERROR(I10,"")</f>
         <v/>
       </c>
-      <c r="L10" s="17" t="n"/>
-      <c r="M10" s="27" t="n"/>
+      <c r="L10" s="17" t="n">
+        <v>1940.8</v>
+      </c>
+      <c r="M10" s="27" t="n">
+        <v>400</v>
+      </c>
       <c r="N10" s="31">
         <f>IFERROR(G10+M10,"")</f>
         <v/>
@@ -11204,19 +11228,31 @@
       <c r="Q9" s="32" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="33" t="n"/>
-      <c r="B10" s="15" t="n"/>
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="n">
+        <v>6</v>
+      </c>
       <c r="C10" s="7">
         <f>IFERROR(参数配置!$C$6*(B10-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D10" s="27" t="n"/>
-      <c r="E10" s="27" t="n"/>
+      <c r="D10" s="27" t="n">
+        <v>8.843999999999999</v>
+      </c>
+      <c r="E10" s="27" t="n">
+        <v>7.342891065597534</v>
+      </c>
       <c r="F10" s="28">
         <f>IFERROR((D10-E10)/E10,"")</f>
         <v/>
       </c>
-      <c r="G10" s="27" t="n"/>
+      <c r="G10" s="27" t="n">
+        <v>900</v>
+      </c>
       <c r="H10" s="7">
         <f>IFERROR(G10*D10,"")</f>
         <v/>
@@ -11233,8 +11269,12 @@
         <f>IFERROR(I10,"")</f>
         <v/>
       </c>
-      <c r="L10" s="17" t="n"/>
-      <c r="M10" s="27" t="n"/>
+      <c r="L10" s="17" t="n">
+        <v>884.4</v>
+      </c>
+      <c r="M10" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="N10" s="31">
         <f>IFERROR(G10+M10,"")</f>
         <v/>
@@ -16061,19 +16101,31 @@
       <c r="Q9" s="32" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="33" t="n"/>
-      <c r="B10" s="15" t="n"/>
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="n">
+        <v>6</v>
+      </c>
       <c r="C10" s="7">
         <f>IFERROR(参数配置!$C$7*(B10-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D10" s="27" t="n"/>
-      <c r="E10" s="27" t="n"/>
+      <c r="D10" s="27" t="n">
+        <v>1.382</v>
+      </c>
+      <c r="E10" s="27" t="n">
+        <v>1.553168001651764</v>
+      </c>
       <c r="F10" s="28">
         <f>IFERROR((D10-E10)/E10,"")</f>
         <v/>
       </c>
-      <c r="G10" s="27" t="n"/>
+      <c r="G10" s="27" t="n">
+        <v>2200</v>
+      </c>
       <c r="H10" s="7">
         <f>IFERROR(G10*D10,"")</f>
         <v/>
@@ -16090,8 +16142,12 @@
         <f>IFERROR(I10,"")</f>
         <v/>
       </c>
-      <c r="L10" s="17" t="n"/>
-      <c r="M10" s="27" t="n"/>
+      <c r="L10" s="17" t="n">
+        <v>552.8</v>
+      </c>
+      <c r="M10" s="27" t="n">
+        <v>400</v>
+      </c>
       <c r="N10" s="31">
         <f>IFERROR(G10+M10,"")</f>
         <v/>
@@ -20922,19 +20978,31 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="33" t="n"/>
-      <c r="B10" s="15" t="n"/>
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="n">
+        <v>6</v>
+      </c>
       <c r="C10" s="7">
         <f>IFERROR(参数配置!$C$8*(B10-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D10" s="27" t="n"/>
-      <c r="E10" s="27" t="n"/>
+      <c r="D10" s="27" t="n">
+        <v>2.149</v>
+      </c>
+      <c r="E10" s="27" t="n">
+        <v>1.814727995872498</v>
+      </c>
       <c r="F10" s="28">
         <f>IFERROR((D10-E10)/E10,"")</f>
         <v/>
       </c>
-      <c r="G10" s="27" t="n"/>
+      <c r="G10" s="27" t="n">
+        <v>4400</v>
+      </c>
       <c r="H10" s="7">
         <f>IFERROR(G10*D10,"")</f>
         <v/>
@@ -20951,8 +21019,12 @@
         <f>IFERROR(I10,"")</f>
         <v/>
       </c>
-      <c r="L10" s="17" t="n"/>
-      <c r="M10" s="27" t="n"/>
+      <c r="L10" s="17" t="n">
+        <v>4727.8</v>
+      </c>
+      <c r="M10" s="27" t="n">
+        <v>2200</v>
+      </c>
       <c r="N10" s="31">
         <f>IFERROR(G10+M10,"")</f>
         <v/>

</xml_diff>

<commit_message>
Record DCA periods 7-8.
Period 8 includes a Nasdaq halt with no trade while target value still advances.
</commit_message>
<xml_diff>
--- a/strategies/constant_value/定投追踪记录.xlsx
+++ b/strategies/constant_value/定投追踪记录.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="汇总看板" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="每期汇总" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="参数配置" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="沪深300" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="中证500" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="恒生指数" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="纳指100" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总看板" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每期汇总" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数配置" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="沪深300" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="中证500" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="恒生指数" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="纳指100" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1363,8 +1363,14 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="n"/>
-      <c r="B11" s="33" t="n"/>
+      <c r="A11" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="33" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
       <c r="C11" s="7">
         <f>IFERROR(SUMIF(沪深300!$B$5:$B$1000,A11,沪深300!$L$5:$L$1000),"")</f>
         <v/>
@@ -1385,7 +1391,9 @@
         <f>IFERROR(IF(M11="增量阶段",H11,SUMPRODUCT(MAX(C11,0),1)+SUMPRODUCT(MAX(D11,0),1)+SUMPRODUCT(MAX(E11,0),1)+SUMPRODUCT(MAX(F11,0),1)),"")</f>
         <v/>
       </c>
-      <c r="H11" s="17" t="n"/>
+      <c r="H11" s="17" t="n">
+        <v>0</v>
+      </c>
       <c r="I11" s="7">
         <f>IFERROR(MAX(-C11,0)+MAX(-D11,0)+MAX(-E11,0)+MAX(-F11,0),"")</f>
         <v/>
@@ -1408,8 +1416,14 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="n"/>
-      <c r="B12" s="33" t="n"/>
+      <c r="A12" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="33" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
       <c r="C12" s="7">
         <f>IFERROR(SUMIF(沪深300!$B$5:$B$1000,A12,沪深300!$L$5:$L$1000),"")</f>
         <v/>
@@ -1430,7 +1444,9 @@
         <f>IFERROR(IF(M12="增量阶段",H12,SUMPRODUCT(MAX(C12,0),1)+SUMPRODUCT(MAX(D12,0),1)+SUMPRODUCT(MAX(E12,0),1)+SUMPRODUCT(MAX(F12,0),1)),"")</f>
         <v/>
       </c>
-      <c r="H12" s="17" t="n"/>
+      <c r="H12" s="17" t="n">
+        <v>0</v>
+      </c>
       <c r="I12" s="7">
         <f>IFERROR(MAX(-C12,0)+MAX(-D12,0)+MAX(-E12,0)+MAX(-F12,0),"")</f>
         <v/>
@@ -6417,19 +6433,31 @@
       <c r="Q10" s="32" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="33" t="n"/>
-      <c r="B11" s="15" t="n"/>
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="n">
+        <v>7</v>
+      </c>
       <c r="C11" s="7">
         <f>IFERROR(参数配置!$C$5*(B11-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D11" s="27" t="n"/>
-      <c r="E11" s="27" t="n"/>
+      <c r="D11" s="27" t="n">
+        <v>4.643</v>
+      </c>
+      <c r="E11" s="27" t="n">
+        <v>4.598508</v>
+      </c>
       <c r="F11" s="28">
         <f>IFERROR((D11-E11)/E11,"")</f>
         <v/>
       </c>
-      <c r="G11" s="27" t="n"/>
+      <c r="G11" s="27" t="n">
+        <v>1900</v>
+      </c>
       <c r="H11" s="7">
         <f>IFERROR(G11*D11,"")</f>
         <v/>
@@ -6446,8 +6474,12 @@
         <f>IFERROR(I11,"")</f>
         <v/>
       </c>
-      <c r="L11" s="17" t="n"/>
-      <c r="M11" s="27" t="n"/>
+      <c r="L11" s="17" t="n">
+        <v>1857.2</v>
+      </c>
+      <c r="M11" s="27" t="n">
+        <v>400</v>
+      </c>
       <c r="N11" s="31">
         <f>IFERROR(G11+M11,"")</f>
         <v/>
@@ -6463,19 +6495,31 @@
       <c r="Q11" s="32" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="33" t="n"/>
-      <c r="B12" s="15" t="n"/>
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="n">
+        <v>8</v>
+      </c>
       <c r="C12" s="7">
         <f>IFERROR(参数配置!$C$5*(B12-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D12" s="27" t="n"/>
-      <c r="E12" s="27" t="n"/>
+      <c r="D12" s="27" t="n">
+        <v>4.691</v>
+      </c>
+      <c r="E12" s="27" t="n">
+        <v>4.6278</v>
+      </c>
       <c r="F12" s="28">
         <f>IFERROR((D12-E12)/E12,"")</f>
         <v/>
       </c>
-      <c r="G12" s="27" t="n"/>
+      <c r="G12" s="27" t="n">
+        <v>2300</v>
+      </c>
       <c r="H12" s="7">
         <f>IFERROR(G12*D12,"")</f>
         <v/>
@@ -6492,8 +6536,12 @@
         <f>IFERROR(I12,"")</f>
         <v/>
       </c>
-      <c r="L12" s="17" t="n"/>
-      <c r="M12" s="27" t="n"/>
+      <c r="L12" s="17" t="n">
+        <v>1407.3</v>
+      </c>
+      <c r="M12" s="27" t="n">
+        <v>300</v>
+      </c>
       <c r="N12" s="31">
         <f>IFERROR(G12+M12,"")</f>
         <v/>
@@ -11290,19 +11338,31 @@
       <c r="Q10" s="32" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="33" t="n"/>
-      <c r="B11" s="15" t="n"/>
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="n">
+        <v>7</v>
+      </c>
       <c r="C11" s="7">
         <f>IFERROR(参数配置!$C$6*(B11-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D11" s="27" t="n"/>
-      <c r="E11" s="27" t="n"/>
+      <c r="D11" s="27" t="n">
+        <v>7.728</v>
+      </c>
+      <c r="E11" s="27" t="n">
+        <v>7.549152</v>
+      </c>
       <c r="F11" s="28">
         <f>IFERROR((D11-E11)/E11,"")</f>
         <v/>
       </c>
-      <c r="G11" s="27" t="n"/>
+      <c r="G11" s="27" t="n">
+        <v>1000</v>
+      </c>
       <c r="H11" s="7">
         <f>IFERROR(G11*D11,"")</f>
         <v/>
@@ -11319,8 +11379,12 @@
         <f>IFERROR(I11,"")</f>
         <v/>
       </c>
-      <c r="L11" s="17" t="n"/>
-      <c r="M11" s="27" t="n"/>
+      <c r="L11" s="17" t="n">
+        <v>2318.4</v>
+      </c>
+      <c r="M11" s="27" t="n">
+        <v>300</v>
+      </c>
       <c r="N11" s="31">
         <f>IFERROR(G11+M11,"")</f>
         <v/>
@@ -11336,19 +11400,31 @@
       <c r="Q11" s="32" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="33" t="n"/>
-      <c r="B12" s="15" t="n"/>
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="n">
+        <v>8</v>
+      </c>
       <c r="C12" s="7">
         <f>IFERROR(参数配置!$C$6*(B12-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D12" s="27" t="n"/>
-      <c r="E12" s="27" t="n"/>
+      <c r="D12" s="27" t="n">
+        <v>7.63</v>
+      </c>
+      <c r="E12" s="27" t="n">
+        <v>7.6165</v>
+      </c>
       <c r="F12" s="28">
         <f>IFERROR((D12-E12)/E12,"")</f>
         <v/>
       </c>
-      <c r="G12" s="27" t="n"/>
+      <c r="G12" s="27" t="n">
+        <v>1300</v>
+      </c>
       <c r="H12" s="7">
         <f>IFERROR(G12*D12,"")</f>
         <v/>
@@ -11365,8 +11441,12 @@
         <f>IFERROR(I12,"")</f>
         <v/>
       </c>
-      <c r="L12" s="17" t="n"/>
-      <c r="M12" s="27" t="n"/>
+      <c r="L12" s="17" t="n">
+        <v>1526</v>
+      </c>
+      <c r="M12" s="27" t="n">
+        <v>200</v>
+      </c>
       <c r="N12" s="31">
         <f>IFERROR(G12+M12,"")</f>
         <v/>
@@ -16163,19 +16243,31 @@
       <c r="Q10" s="32" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="33" t="n"/>
-      <c r="B11" s="15" t="n"/>
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="n">
+        <v>7</v>
+      </c>
       <c r="C11" s="7">
         <f>IFERROR(参数配置!$C$7*(B11-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D11" s="27" t="n"/>
-      <c r="E11" s="27" t="n"/>
+      <c r="D11" s="27" t="n">
+        <v>1.462</v>
+      </c>
+      <c r="E11" s="27" t="n">
+        <v>1.548248</v>
+      </c>
       <c r="F11" s="28">
         <f>IFERROR((D11-E11)/E11,"")</f>
         <v/>
       </c>
-      <c r="G11" s="27" t="n"/>
+      <c r="G11" s="27" t="n">
+        <v>2600</v>
+      </c>
       <c r="H11" s="7">
         <f>IFERROR(G11*D11,"")</f>
         <v/>
@@ -16192,8 +16284,12 @@
         <f>IFERROR(I11,"")</f>
         <v/>
       </c>
-      <c r="L11" s="17" t="n"/>
-      <c r="M11" s="27" t="n"/>
+      <c r="L11" s="17" t="n">
+        <v>438.6</v>
+      </c>
+      <c r="M11" s="27" t="n">
+        <v>300</v>
+      </c>
       <c r="N11" s="31">
         <f>IFERROR(G11+M11,"")</f>
         <v/>
@@ -16209,19 +16305,31 @@
       <c r="Q11" s="32" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="33" t="n"/>
-      <c r="B12" s="15" t="n"/>
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="n">
+        <v>8</v>
+      </c>
       <c r="C12" s="7">
         <f>IFERROR(参数配置!$C$7*(B12-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D12" s="27" t="n"/>
-      <c r="E12" s="27" t="n"/>
+      <c r="D12" s="27" t="n">
+        <v>1.523</v>
+      </c>
+      <c r="E12" s="27" t="n">
+        <v>1.5482</v>
+      </c>
       <c r="F12" s="28">
         <f>IFERROR((D12-E12)/E12,"")</f>
         <v/>
       </c>
-      <c r="G12" s="27" t="n"/>
+      <c r="G12" s="27" t="n">
+        <v>2900</v>
+      </c>
       <c r="H12" s="7">
         <f>IFERROR(G12*D12,"")</f>
         <v/>
@@ -16238,8 +16346,12 @@
         <f>IFERROR(I12,"")</f>
         <v/>
       </c>
-      <c r="L12" s="17" t="n"/>
-      <c r="M12" s="27" t="n"/>
+      <c r="L12" s="17" t="n">
+        <v>304.6</v>
+      </c>
+      <c r="M12" s="27" t="n">
+        <v>200</v>
+      </c>
       <c r="N12" s="31">
         <f>IFERROR(G12+M12,"")</f>
         <v/>
@@ -21040,19 +21152,31 @@
       <c r="Q10" s="32" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="33" t="n"/>
-      <c r="B11" s="15" t="n"/>
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="n">
+        <v>7</v>
+      </c>
       <c r="C11" s="7">
         <f>IFERROR(参数配置!$C$8*(B11-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D11" s="27" t="n"/>
-      <c r="E11" s="27" t="n"/>
+      <c r="D11" s="27" t="n">
+        <v>2.117</v>
+      </c>
+      <c r="E11" s="27" t="n">
+        <v>1.890264</v>
+      </c>
       <c r="F11" s="28">
         <f>IFERROR((D11-E11)/E11,"")</f>
         <v/>
       </c>
-      <c r="G11" s="27" t="n"/>
+      <c r="G11" s="27" t="n">
+        <v>6600</v>
+      </c>
       <c r="H11" s="7">
         <f>IFERROR(G11*D11,"")</f>
         <v/>
@@ -21069,8 +21193,12 @@
         <f>IFERROR(I11,"")</f>
         <v/>
       </c>
-      <c r="L11" s="17" t="n"/>
-      <c r="M11" s="27" t="n"/>
+      <c r="L11" s="17" t="n">
+        <v>2752.1</v>
+      </c>
+      <c r="M11" s="27" t="n">
+        <v>1300</v>
+      </c>
       <c r="N11" s="31">
         <f>IFERROR(G11+M11,"")</f>
         <v/>
@@ -21086,19 +21214,31 @@
       <c r="Q11" s="32" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="33" t="n"/>
-      <c r="B12" s="15" t="n"/>
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="n">
+        <v>8</v>
+      </c>
       <c r="C12" s="7">
         <f>IFERROR(参数配置!$C$8*(B12-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D12" s="27" t="n"/>
-      <c r="E12" s="27" t="n"/>
+      <c r="D12" s="27" t="n">
+        <v>2.117</v>
+      </c>
+      <c r="E12" s="27" t="n">
+        <v>1.9067</v>
+      </c>
       <c r="F12" s="28">
         <f>IFERROR((D12-E12)/E12,"")</f>
         <v/>
       </c>
-      <c r="G12" s="27" t="n"/>
+      <c r="G12" s="27" t="n">
+        <v>7900</v>
+      </c>
       <c r="H12" s="7">
         <f>IFERROR(G12*D12,"")</f>
         <v/>
@@ -21115,8 +21255,12 @@
         <f>IFERROR(I12,"")</f>
         <v/>
       </c>
-      <c r="L12" s="17" t="n"/>
-      <c r="M12" s="27" t="n"/>
+      <c r="L12" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="N12" s="31">
         <f>IFERROR(G12+M12,"")</f>
         <v/>
@@ -21129,7 +21273,11 @@
         <f>IFERROR(-L12,"")</f>
         <v/>
       </c>
-      <c r="Q12" s="32" t="n"/>
+      <c r="Q12" s="32" t="inlineStr">
+        <is>
+          <t>停牌，本期暂停操作，目标市值照常增长</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="33" t="n"/>

</xml_diff>

<commit_message>
Record DCA period 9.
Nasdaq resumes after the period-8 halt; other ETFs continue regular buys.
</commit_message>
<xml_diff>
--- a/strategies/constant_value/定投追踪记录.xlsx
+++ b/strategies/constant_value/定投追踪记录.xlsx
@@ -1469,8 +1469,14 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="n"/>
-      <c r="B13" s="33" t="n"/>
+      <c r="A13" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="33" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
       <c r="C13" s="7">
         <f>IFERROR(SUMIF(沪深300!$B$5:$B$1000,A13,沪深300!$L$5:$L$1000),"")</f>
         <v/>
@@ -1491,7 +1497,9 @@
         <f>IFERROR(IF(M13="增量阶段",H13,SUMPRODUCT(MAX(C13,0),1)+SUMPRODUCT(MAX(D13,0),1)+SUMPRODUCT(MAX(E13,0),1)+SUMPRODUCT(MAX(F13,0),1)),"")</f>
         <v/>
       </c>
-      <c r="H13" s="17" t="n"/>
+      <c r="H13" s="17" t="n">
+        <v>0</v>
+      </c>
       <c r="I13" s="7">
         <f>IFERROR(MAX(-C13,0)+MAX(-D13,0)+MAX(-E13,0)+MAX(-F13,0),"")</f>
         <v/>
@@ -6557,19 +6565,31 @@
       <c r="Q12" s="32" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="33" t="n"/>
-      <c r="B13" s="15" t="n"/>
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="n">
+        <v>9</v>
+      </c>
       <c r="C13" s="7">
         <f>IFERROR(参数配置!$C$5*(B13-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D13" s="27" t="n"/>
-      <c r="E13" s="27" t="n"/>
+      <c r="D13" s="27" t="n">
+        <v>4.724</v>
+      </c>
+      <c r="E13" s="27" t="n">
+        <v>4.6531</v>
+      </c>
       <c r="F13" s="28">
         <f>IFERROR((D13-E13)/E13,"")</f>
         <v/>
       </c>
-      <c r="G13" s="27" t="n"/>
+      <c r="G13" s="27" t="n">
+        <v>2600</v>
+      </c>
       <c r="H13" s="7">
         <f>IFERROR(G13*D13,"")</f>
         <v/>
@@ -6586,8 +6606,12 @@
         <f>IFERROR(I13,"")</f>
         <v/>
       </c>
-      <c r="L13" s="17" t="n"/>
-      <c r="M13" s="27" t="n"/>
+      <c r="L13" s="17" t="n">
+        <v>944.8000000000001</v>
+      </c>
+      <c r="M13" s="27" t="n">
+        <v>200</v>
+      </c>
       <c r="N13" s="31">
         <f>IFERROR(G13+M13,"")</f>
         <v/>
@@ -11462,19 +11486,31 @@
       <c r="Q12" s="32" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="33" t="n"/>
-      <c r="B13" s="15" t="n"/>
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="n">
+        <v>9</v>
+      </c>
       <c r="C13" s="7">
         <f>IFERROR(参数配置!$C$6*(B13-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D13" s="27" t="n"/>
-      <c r="E13" s="27" t="n"/>
+      <c r="D13" s="27" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="E13" s="27" t="n">
+        <v>7.6852</v>
+      </c>
       <c r="F13" s="28">
         <f>IFERROR((D13-E13)/E13,"")</f>
         <v/>
       </c>
-      <c r="G13" s="27" t="n"/>
+      <c r="G13" s="27" t="n">
+        <v>1500</v>
+      </c>
       <c r="H13" s="7">
         <f>IFERROR(G13*D13,"")</f>
         <v/>
@@ -11491,8 +11527,12 @@
         <f>IFERROR(I13,"")</f>
         <v/>
       </c>
-      <c r="L13" s="17" t="n"/>
-      <c r="M13" s="27" t="n"/>
+      <c r="L13" s="17" t="n">
+        <v>1598</v>
+      </c>
+      <c r="M13" s="27" t="n">
+        <v>200</v>
+      </c>
       <c r="N13" s="31">
         <f>IFERROR(G13+M13,"")</f>
         <v/>
@@ -16367,19 +16407,31 @@
       <c r="Q12" s="32" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="33" t="n"/>
-      <c r="B13" s="15" t="n"/>
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="n">
+        <v>9</v>
+      </c>
       <c r="C13" s="7">
         <f>IFERROR(参数配置!$C$7*(B13-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D13" s="27" t="n"/>
-      <c r="E13" s="27" t="n"/>
+      <c r="D13" s="27" t="n">
+        <v>1.479</v>
+      </c>
+      <c r="E13" s="27" t="n">
+        <v>1.5466</v>
+      </c>
       <c r="F13" s="28">
         <f>IFERROR((D13-E13)/E13,"")</f>
         <v/>
       </c>
-      <c r="G13" s="27" t="n"/>
+      <c r="G13" s="27" t="n">
+        <v>3100</v>
+      </c>
       <c r="H13" s="7">
         <f>IFERROR(G13*D13,"")</f>
         <v/>
@@ -16396,8 +16448,12 @@
         <f>IFERROR(I13,"")</f>
         <v/>
       </c>
-      <c r="L13" s="17" t="n"/>
-      <c r="M13" s="27" t="n"/>
+      <c r="L13" s="17" t="n">
+        <v>739.5</v>
+      </c>
+      <c r="M13" s="27" t="n">
+        <v>500</v>
+      </c>
       <c r="N13" s="31">
         <f>IFERROR(G13+M13,"")</f>
         <v/>
@@ -21280,19 +21336,31 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="33" t="n"/>
-      <c r="B13" s="15" t="n"/>
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="n">
+        <v>9</v>
+      </c>
       <c r="C13" s="7">
         <f>IFERROR(参数配置!$C$8*(B13-$S$3),"")</f>
         <v/>
       </c>
-      <c r="D13" s="27" t="n"/>
-      <c r="E13" s="27" t="n"/>
+      <c r="D13" s="27" t="n">
+        <v>2.264</v>
+      </c>
+      <c r="E13" s="27" t="n">
+        <v>1.9307</v>
+      </c>
       <c r="F13" s="28">
         <f>IFERROR((D13-E13)/E13,"")</f>
         <v/>
       </c>
-      <c r="G13" s="27" t="n"/>
+      <c r="G13" s="27" t="n">
+        <v>7900</v>
+      </c>
       <c r="H13" s="7">
         <f>IFERROR(G13*D13,"")</f>
         <v/>
@@ -21309,8 +21377,12 @@
         <f>IFERROR(I13,"")</f>
         <v/>
       </c>
-      <c r="L13" s="17" t="n"/>
-      <c r="M13" s="27" t="n"/>
+      <c r="L13" s="17" t="n">
+        <v>3622.4</v>
+      </c>
+      <c r="M13" s="27" t="n">
+        <v>1600</v>
+      </c>
       <c r="N13" s="31">
         <f>IFERROR(G13+M13,"")</f>
         <v/>

</xml_diff>